<commit_message>
feat(voice-agent): enhance UI and percentile mapping
- Migrate to Groq Whisper STT for universal browser support
- Implement Voice Activity Detection (VAD) for hands-free auto-stop
- Add Missing Fields smart card visual payload, removing TTS text wall
- Fix CAT percentile linear scaling bug by adding exponential raw score mapping
- Update all institute calculators to accurately map scaled CAT components
- Refactor Landing Page to highlight Clymber Voice Agent in Hero Section
</commit_message>
<xml_diff>
--- a/Dataset/mba_admissions_benchmark_reconstruction_v4.xlsx
+++ b/Dataset/mba_admissions_benchmark_reconstruction_v4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Clymber\voice-agent\Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C69057-9E48-439D-807D-ED097C3B2F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C7625E-58A2-4A2B-9A3D-CC9E9DB311A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3138,17 +3138,17 @@
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
       <c r="C2">
-        <v>89.35</v>
+        <v>89.55</v>
       </c>
       <c r="D2">
-        <v>91.75</v>
+        <v>91.95</v>
       </c>
       <c r="E2">
-        <v>94.15</v>
+        <v>94.350000000000009</v>
       </c>
       <c r="F2" s="3">
         <v>99.62</v>
@@ -3170,17 +3170,17 @@
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>13</v>
       </c>
       <c r="C3">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D3">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E3">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F3" s="3">
         <v>99.15</v>
@@ -3202,17 +3202,17 @@
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>15</v>
       </c>
       <c r="C4">
-        <v>83.95</v>
+        <v>84.15</v>
       </c>
       <c r="D4">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="E4">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="F4" s="3">
         <v>98.3</v>
@@ -3234,17 +3234,17 @@
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
-        <v>75.150000000000006</v>
+        <v>75.350000000000009</v>
       </c>
       <c r="D5">
-        <v>79.75</v>
+        <v>79.95</v>
       </c>
       <c r="E5">
-        <v>84.35</v>
+        <v>84.55</v>
       </c>
       <c r="F5" s="3">
         <v>91</v>
@@ -3266,17 +3266,17 @@
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
       <c r="C6">
-        <v>69.150000000000006</v>
+        <v>69.350000000000009</v>
       </c>
       <c r="D6">
-        <v>74.75</v>
+        <v>74.95</v>
       </c>
       <c r="E6">
-        <v>80.849999999999994</v>
+        <v>81.05</v>
       </c>
       <c r="F6" s="3">
         <v>81</v>
@@ -3298,17 +3298,17 @@
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
       <c r="C7">
-        <v>67.650000000000006</v>
+        <v>67.850000000000009</v>
       </c>
       <c r="D7">
-        <v>73.25</v>
+        <v>73.45</v>
       </c>
       <c r="E7">
-        <v>79.349999999999994</v>
+        <v>79.55</v>
       </c>
       <c r="F7" s="3">
         <v>76</v>
@@ -3330,17 +3330,17 @@
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8">
-        <v>89.05</v>
+        <v>89.25</v>
       </c>
       <c r="D8">
-        <v>91.45</v>
+        <v>91.65</v>
       </c>
       <c r="E8">
-        <v>93.85</v>
+        <v>94.05</v>
       </c>
       <c r="F8" s="3">
         <v>99.45</v>
@@ -3362,17 +3362,17 @@
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>13</v>
       </c>
       <c r="C9">
-        <v>86.65</v>
+        <v>86.850000000000009</v>
       </c>
       <c r="D9">
-        <v>89.45</v>
+        <v>89.65</v>
       </c>
       <c r="E9">
-        <v>92.25</v>
+        <v>92.45</v>
       </c>
       <c r="F9" s="3">
         <v>98.85</v>
@@ -3394,17 +3394,17 @@
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>15</v>
       </c>
       <c r="C10">
-        <v>83.65</v>
+        <v>83.850000000000009</v>
       </c>
       <c r="D10">
-        <v>86.45</v>
+        <v>86.65</v>
       </c>
       <c r="E10">
-        <v>89.25</v>
+        <v>89.45</v>
       </c>
       <c r="F10" s="3">
         <v>97.8</v>
@@ -3426,17 +3426,17 @@
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>16</v>
       </c>
       <c r="C11">
-        <v>74.849999999999994</v>
+        <v>75.05</v>
       </c>
       <c r="D11">
-        <v>79.45</v>
+        <v>79.650000000000006</v>
       </c>
       <c r="E11">
-        <v>84.05</v>
+        <v>84.25</v>
       </c>
       <c r="F11" s="3">
         <v>89.5</v>
@@ -3458,17 +3458,17 @@
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>18</v>
       </c>
       <c r="C12">
-        <v>68.849999999999994</v>
+        <v>69.05</v>
       </c>
       <c r="D12">
-        <v>74.45</v>
+        <v>74.650000000000006</v>
       </c>
       <c r="E12">
-        <v>80.55</v>
+        <v>80.75</v>
       </c>
       <c r="F12" s="3">
         <v>80</v>
@@ -3490,17 +3490,17 @@
       <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>20</v>
       </c>
       <c r="C13">
-        <v>67.349999999999994</v>
+        <v>67.55</v>
       </c>
       <c r="D13">
-        <v>72.95</v>
+        <v>73.150000000000006</v>
       </c>
       <c r="E13">
-        <v>79.05</v>
+        <v>79.25</v>
       </c>
       <c r="F13" s="3">
         <v>74</v>
@@ -3522,17 +3522,17 @@
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>11</v>
       </c>
       <c r="C14">
-        <v>89.15</v>
+        <v>89.350000000000009</v>
       </c>
       <c r="D14">
-        <v>91.55</v>
+        <v>91.75</v>
       </c>
       <c r="E14">
-        <v>93.95</v>
+        <v>94.15</v>
       </c>
       <c r="F14" s="3">
         <v>99.55</v>
@@ -3554,17 +3554,17 @@
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>13</v>
       </c>
       <c r="C15">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D15">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E15">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F15" s="3">
         <v>99</v>
@@ -3586,17 +3586,17 @@
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>15</v>
       </c>
       <c r="C16">
-        <v>83.75</v>
+        <v>83.95</v>
       </c>
       <c r="D16">
-        <v>86.55</v>
+        <v>86.75</v>
       </c>
       <c r="E16">
-        <v>89.35</v>
+        <v>89.55</v>
       </c>
       <c r="F16" s="3">
         <v>98.1</v>
@@ -3618,17 +3618,17 @@
       <c r="A17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" t="s">
         <v>16</v>
       </c>
       <c r="C17">
-        <v>74.95</v>
+        <v>75.150000000000006</v>
       </c>
       <c r="D17">
-        <v>79.55</v>
+        <v>79.75</v>
       </c>
       <c r="E17">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="F17" s="3">
         <v>90</v>
@@ -3650,17 +3650,17 @@
       <c r="A18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18">
-        <v>68.95</v>
+        <v>69.150000000000006</v>
       </c>
       <c r="D18">
-        <v>74.55</v>
+        <v>74.75</v>
       </c>
       <c r="E18">
-        <v>80.650000000000006</v>
+        <v>80.850000000000009</v>
       </c>
       <c r="F18" s="3">
         <v>80.5</v>
@@ -3682,17 +3682,17 @@
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" t="s">
         <v>20</v>
       </c>
       <c r="C19">
-        <v>67.45</v>
+        <v>67.650000000000006</v>
       </c>
       <c r="D19">
-        <v>73.05</v>
+        <v>73.25</v>
       </c>
       <c r="E19">
-        <v>79.150000000000006</v>
+        <v>79.350000000000009</v>
       </c>
       <c r="F19" s="3">
         <v>75</v>
@@ -3714,17 +3714,17 @@
       <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" t="s">
         <v>11</v>
       </c>
       <c r="C20">
-        <v>46.75</v>
+        <v>46.95</v>
       </c>
       <c r="D20">
-        <v>50.25</v>
+        <v>50.45</v>
       </c>
       <c r="E20">
-        <v>53.75</v>
+        <v>53.95</v>
       </c>
       <c r="F20" s="3">
         <v>99.5</v>
@@ -3746,17 +3746,17 @@
       <c r="A21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" t="s">
         <v>13</v>
       </c>
       <c r="C21">
-        <v>37.15</v>
+        <v>37.35</v>
       </c>
       <c r="D21">
-        <v>39.950000000000003</v>
+        <v>40.150000000000006</v>
       </c>
       <c r="E21">
-        <v>42.95</v>
+        <v>43.150000000000006</v>
       </c>
       <c r="F21" s="3">
         <v>98.9</v>
@@ -3778,17 +3778,17 @@
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" t="s">
         <v>15</v>
       </c>
       <c r="C22">
-        <v>35.25</v>
+        <v>35.450000000000003</v>
       </c>
       <c r="D22">
-        <v>38.549999999999997</v>
+        <v>38.75</v>
       </c>
       <c r="E22">
-        <v>41.75</v>
+        <v>41.95</v>
       </c>
       <c r="F22" s="3">
         <v>97.5</v>
@@ -3810,17 +3810,17 @@
       <c r="A23" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" t="s">
         <v>16</v>
       </c>
       <c r="C23">
-        <v>28.75</v>
+        <v>28.95</v>
       </c>
       <c r="D23">
-        <v>31.75</v>
+        <v>31.95</v>
       </c>
       <c r="E23">
-        <v>34.75</v>
+        <v>34.950000000000003</v>
       </c>
       <c r="F23" s="3">
         <v>86</v>
@@ -3842,17 +3842,17 @@
       <c r="A24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" t="s">
         <v>18</v>
       </c>
       <c r="C24">
-        <v>21.25</v>
+        <v>21.45</v>
       </c>
       <c r="D24">
-        <v>24.75</v>
+        <v>24.95</v>
       </c>
       <c r="E24">
-        <v>28.75</v>
+        <v>28.95</v>
       </c>
       <c r="F24" s="3">
         <v>78.5</v>
@@ -3874,17 +3874,17 @@
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" t="s">
         <v>20</v>
       </c>
       <c r="C25">
-        <v>23.75</v>
+        <v>23.95</v>
       </c>
       <c r="D25">
-        <v>27.25</v>
+        <v>27.45</v>
       </c>
       <c r="E25">
-        <v>30.75</v>
+        <v>30.95</v>
       </c>
       <c r="F25" s="3">
         <v>70</v>
@@ -3906,17 +3906,17 @@
       <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" t="s">
         <v>11</v>
       </c>
       <c r="C26">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D26">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E26">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F26" s="3">
         <v>96</v>
@@ -3938,17 +3938,17 @@
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" t="s">
         <v>13</v>
       </c>
       <c r="C27">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D27">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E27">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F27" s="3">
         <v>96</v>
@@ -3970,17 +3970,17 @@
       <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" t="s">
         <v>15</v>
       </c>
       <c r="C28">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D28">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E28">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F28" s="3">
         <v>96</v>
@@ -4002,17 +4002,17 @@
       <c r="A29" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" t="s">
         <v>16</v>
       </c>
       <c r="C29">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D29">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E29">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F29" s="3">
         <v>96</v>
@@ -4034,17 +4034,17 @@
       <c r="A30" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" t="s">
         <v>18</v>
       </c>
       <c r="C30">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D30">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E30">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F30" s="3">
         <v>96</v>
@@ -4066,17 +4066,17 @@
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" t="s">
         <v>20</v>
       </c>
       <c r="C31">
-        <v>88.55</v>
+        <v>88.75</v>
       </c>
       <c r="D31">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="E31">
-        <v>93.35</v>
+        <v>93.55</v>
       </c>
       <c r="F31" s="3">
         <v>96</v>
@@ -4098,17 +4098,17 @@
       <c r="A32" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" t="s">
         <v>11</v>
       </c>
       <c r="C32">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D32">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E32">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F32" s="3">
         <v>97.5</v>
@@ -4130,17 +4130,17 @@
       <c r="A33" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" t="s">
         <v>13</v>
       </c>
       <c r="C33">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D33">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E33">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F33" s="3">
         <v>97.5</v>
@@ -4162,17 +4162,17 @@
       <c r="A34" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" t="s">
         <v>15</v>
       </c>
       <c r="C34">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D34">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E34">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F34" s="3">
         <v>97.5</v>
@@ -4194,17 +4194,17 @@
       <c r="A35" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" t="s">
         <v>16</v>
       </c>
       <c r="C35">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D35">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E35">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F35" s="3">
         <v>97.5</v>
@@ -4226,17 +4226,17 @@
       <c r="A36" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" t="s">
         <v>18</v>
       </c>
       <c r="C36">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D36">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E36">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F36" s="3">
         <v>97.5</v>
@@ -4258,17 +4258,17 @@
       <c r="A37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" t="s">
         <v>20</v>
       </c>
       <c r="C37">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="D37">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="E37">
-        <v>92.15</v>
+        <v>92.350000000000009</v>
       </c>
       <c r="F37" s="3">
         <v>97.5</v>
@@ -4290,17 +4290,17 @@
       <c r="A38" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" t="s">
         <v>11</v>
       </c>
       <c r="C38">
-        <v>87.55</v>
+        <v>87.75</v>
       </c>
       <c r="D38">
-        <v>89.95</v>
+        <v>90.15</v>
       </c>
       <c r="E38">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F38" s="3">
         <v>98.9</v>
@@ -4322,17 +4322,17 @@
       <c r="A39" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" t="s">
         <v>13</v>
       </c>
       <c r="C39">
-        <v>85.15</v>
+        <v>85.350000000000009</v>
       </c>
       <c r="D39">
-        <v>87.95</v>
+        <v>88.15</v>
       </c>
       <c r="E39">
-        <v>90.75</v>
+        <v>90.95</v>
       </c>
       <c r="F39" s="3">
         <v>98.2</v>
@@ -4354,17 +4354,17 @@
       <c r="A40" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" t="s">
         <v>15</v>
       </c>
       <c r="C40">
-        <v>81.75</v>
+        <v>81.95</v>
       </c>
       <c r="D40">
-        <v>84.95</v>
+        <v>85.15</v>
       </c>
       <c r="E40">
-        <v>88.15</v>
+        <v>88.350000000000009</v>
       </c>
       <c r="F40" s="3">
         <v>96.7</v>
@@ -4386,17 +4386,17 @@
       <c r="A41" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" t="s">
         <v>16</v>
       </c>
       <c r="C41">
-        <v>73.349999999999994</v>
+        <v>73.55</v>
       </c>
       <c r="D41">
-        <v>77.95</v>
+        <v>78.150000000000006</v>
       </c>
       <c r="E41">
-        <v>82.55</v>
+        <v>82.75</v>
       </c>
       <c r="F41" s="3">
         <v>86.5</v>
@@ -4418,17 +4418,17 @@
       <c r="A42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" t="s">
         <v>18</v>
       </c>
       <c r="C42">
-        <v>67.349999999999994</v>
+        <v>67.55</v>
       </c>
       <c r="D42">
-        <v>72.95</v>
+        <v>73.150000000000006</v>
       </c>
       <c r="E42">
-        <v>79.05</v>
+        <v>79.25</v>
       </c>
       <c r="F42" s="3">
         <v>77</v>
@@ -4450,17 +4450,17 @@
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" t="s">
         <v>20</v>
       </c>
       <c r="C43">
-        <v>65.849999999999994</v>
+        <v>66.05</v>
       </c>
       <c r="D43">
-        <v>71.45</v>
+        <v>71.650000000000006</v>
       </c>
       <c r="E43">
-        <v>77.55</v>
+        <v>77.75</v>
       </c>
       <c r="F43" s="3">
         <v>73</v>
@@ -4482,17 +4482,17 @@
       <c r="A44" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" t="s">
         <v>11</v>
       </c>
       <c r="C44">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D44">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E44">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F44" s="3">
         <v>96.5</v>
@@ -4514,17 +4514,17 @@
       <c r="A45" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" t="s">
         <v>13</v>
       </c>
       <c r="C45">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D45">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E45">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F45" s="3">
         <v>96.5</v>
@@ -4546,17 +4546,17 @@
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" t="s">
         <v>15</v>
       </c>
       <c r="C46">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D46">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E46">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F46" s="3">
         <v>96.5</v>
@@ -4578,17 +4578,17 @@
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" t="s">
         <v>16</v>
       </c>
       <c r="C47">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D47">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E47">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F47" s="3">
         <v>96.5</v>
@@ -4610,17 +4610,17 @@
       <c r="A48" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" t="s">
         <v>18</v>
       </c>
       <c r="C48">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D48">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E48">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F48" s="3">
         <v>96.5</v>
@@ -4642,17 +4642,17 @@
       <c r="A49" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" t="s">
         <v>20</v>
       </c>
       <c r="C49">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="D49">
-        <v>89.55</v>
+        <v>89.75</v>
       </c>
       <c r="E49">
-        <v>92.35</v>
+        <v>92.55</v>
       </c>
       <c r="F49" s="3">
         <v>96.5</v>
@@ -4674,17 +4674,17 @@
       <c r="A50" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" t="s">
         <v>11</v>
       </c>
       <c r="C50">
-        <v>86.35</v>
+        <v>86.55</v>
       </c>
       <c r="D50">
-        <v>89.15</v>
+        <v>89.350000000000009</v>
       </c>
       <c r="E50">
-        <v>91.95</v>
+        <v>92.15</v>
       </c>
       <c r="F50" s="3">
         <v>98.3</v>
@@ -4706,17 +4706,17 @@
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" t="s">
         <v>13</v>
       </c>
       <c r="C51">
-        <v>84.35</v>
+        <v>84.55</v>
       </c>
       <c r="D51">
-        <v>87.15</v>
+        <v>87.350000000000009</v>
       </c>
       <c r="E51">
-        <v>89.95</v>
+        <v>90.15</v>
       </c>
       <c r="F51" s="3">
         <v>97.2</v>
@@ -4738,17 +4738,17 @@
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" t="s">
         <v>15</v>
       </c>
       <c r="C52">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D52">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E52">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F52" s="3">
         <v>94.5</v>
@@ -4770,17 +4770,17 @@
       <c r="A53" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" t="s">
         <v>16</v>
       </c>
       <c r="C53">
-        <v>72.55</v>
+        <v>72.75</v>
       </c>
       <c r="D53">
-        <v>77.150000000000006</v>
+        <v>77.350000000000009</v>
       </c>
       <c r="E53">
-        <v>81.75</v>
+        <v>81.95</v>
       </c>
       <c r="F53" s="3">
         <v>84</v>
@@ -4802,17 +4802,17 @@
       <c r="A54" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" t="s">
         <v>18</v>
       </c>
       <c r="C54">
-        <v>66.55</v>
+        <v>66.75</v>
       </c>
       <c r="D54">
-        <v>72.150000000000006</v>
+        <v>72.350000000000009</v>
       </c>
       <c r="E54">
-        <v>78.25</v>
+        <v>78.45</v>
       </c>
       <c r="F54" s="3">
         <v>75</v>
@@ -4834,17 +4834,17 @@
       <c r="A55" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" t="s">
         <v>20</v>
       </c>
       <c r="C55">
-        <v>65.05</v>
+        <v>65.25</v>
       </c>
       <c r="D55">
-        <v>70.650000000000006</v>
+        <v>70.850000000000009</v>
       </c>
       <c r="E55">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="F55" s="3">
         <v>70</v>
@@ -4866,17 +4866,17 @@
       <c r="A56" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" t="s">
         <v>11</v>
       </c>
       <c r="C56">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D56">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E56">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F56" s="3">
         <v>97.2</v>
@@ -4898,17 +4898,17 @@
       <c r="A57" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" t="s">
         <v>13</v>
       </c>
       <c r="C57">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D57">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E57">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F57" s="3">
         <v>97.2</v>
@@ -4930,17 +4930,17 @@
       <c r="A58" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" t="s">
         <v>15</v>
       </c>
       <c r="C58">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D58">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E58">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F58" s="3">
         <v>97.2</v>
@@ -4962,17 +4962,17 @@
       <c r="A59" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" t="s">
         <v>16</v>
       </c>
       <c r="C59">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D59">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E59">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F59" s="3">
         <v>97.2</v>
@@ -4994,17 +4994,17 @@
       <c r="A60" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" t="s">
         <v>18</v>
       </c>
       <c r="C60">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D60">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E60">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F60" s="3">
         <v>97.2</v>
@@ -5026,17 +5026,17 @@
       <c r="A61" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" t="s">
         <v>20</v>
       </c>
       <c r="C61">
-        <v>85.45</v>
+        <v>85.65</v>
       </c>
       <c r="D61">
-        <v>88.25</v>
+        <v>88.45</v>
       </c>
       <c r="E61">
-        <v>91.05</v>
+        <v>91.25</v>
       </c>
       <c r="F61" s="3">
         <v>97.2</v>
@@ -5058,17 +5058,17 @@
       <c r="A62" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" t="s">
         <v>11</v>
       </c>
       <c r="C62">
-        <v>85.35</v>
+        <v>85.55</v>
       </c>
       <c r="D62">
-        <v>88.15</v>
+        <v>88.350000000000009</v>
       </c>
       <c r="E62">
-        <v>90.95</v>
+        <v>91.15</v>
       </c>
       <c r="F62" s="3">
         <v>97.8</v>
@@ -5090,17 +5090,17 @@
       <c r="A63" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" t="s">
         <v>13</v>
       </c>
       <c r="C63">
-        <v>83.35</v>
+        <v>83.55</v>
       </c>
       <c r="D63">
-        <v>86.15</v>
+        <v>86.350000000000009</v>
       </c>
       <c r="E63">
-        <v>88.95</v>
+        <v>89.15</v>
       </c>
       <c r="F63" s="3">
         <v>96.5</v>
@@ -5122,17 +5122,17 @@
       <c r="A64" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" t="s">
         <v>15</v>
       </c>
       <c r="C64">
-        <v>79.95</v>
+        <v>80.150000000000006</v>
       </c>
       <c r="D64">
-        <v>83.15</v>
+        <v>83.350000000000009</v>
       </c>
       <c r="E64">
-        <v>86.35</v>
+        <v>86.55</v>
       </c>
       <c r="F64" s="3">
         <v>93.5</v>
@@ -5154,17 +5154,17 @@
       <c r="A65" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" t="s">
         <v>16</v>
       </c>
       <c r="C65">
-        <v>71.55</v>
+        <v>71.75</v>
       </c>
       <c r="D65">
-        <v>76.150000000000006</v>
+        <v>76.350000000000009</v>
       </c>
       <c r="E65">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="F65" s="3">
         <v>83.5</v>
@@ -5186,17 +5186,17 @@
       <c r="A66" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" t="s">
         <v>18</v>
       </c>
       <c r="C66">
-        <v>65.55</v>
+        <v>65.75</v>
       </c>
       <c r="D66">
-        <v>71.150000000000006</v>
+        <v>71.350000000000009</v>
       </c>
       <c r="E66">
-        <v>77.25</v>
+        <v>77.45</v>
       </c>
       <c r="F66" s="3">
         <v>74</v>
@@ -5218,17 +5218,17 @@
       <c r="A67" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" t="s">
         <v>20</v>
       </c>
       <c r="C67">
-        <v>63.05</v>
+        <v>63.25</v>
       </c>
       <c r="D67">
-        <v>69.650000000000006</v>
+        <v>69.850000000000009</v>
       </c>
       <c r="E67">
-        <v>77.25</v>
+        <v>77.45</v>
       </c>
       <c r="F67" s="3">
         <v>70</v>
@@ -5250,17 +5250,17 @@
       <c r="A68" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" t="s">
         <v>11</v>
       </c>
       <c r="C68">
-        <v>85.15</v>
+        <v>85.350000000000009</v>
       </c>
       <c r="D68">
-        <v>87.95</v>
+        <v>88.15</v>
       </c>
       <c r="E68">
-        <v>90.75</v>
+        <v>90.95</v>
       </c>
       <c r="F68" s="3">
         <v>99.5</v>
@@ -5282,17 +5282,17 @@
       <c r="A69" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" t="s">
         <v>13</v>
       </c>
       <c r="C69">
-        <v>83.15</v>
+        <v>83.350000000000009</v>
       </c>
       <c r="D69">
-        <v>85.95</v>
+        <v>86.15</v>
       </c>
       <c r="E69">
-        <v>88.75</v>
+        <v>88.95</v>
       </c>
       <c r="F69" s="3">
         <v>99</v>
@@ -5314,17 +5314,17 @@
       <c r="A70" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" t="s">
         <v>15</v>
       </c>
       <c r="C70">
-        <v>79.75</v>
+        <v>79.95</v>
       </c>
       <c r="D70">
-        <v>82.95</v>
+        <v>83.15</v>
       </c>
       <c r="E70">
-        <v>86.15</v>
+        <v>86.350000000000009</v>
       </c>
       <c r="F70" s="3">
         <v>98</v>
@@ -5346,17 +5346,17 @@
       <c r="A71" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" t="s">
         <v>16</v>
       </c>
       <c r="C71">
-        <v>71.349999999999994</v>
+        <v>71.55</v>
       </c>
       <c r="D71">
-        <v>75.95</v>
+        <v>76.150000000000006</v>
       </c>
       <c r="E71">
-        <v>80.55</v>
+        <v>80.75</v>
       </c>
       <c r="F71" s="3">
         <v>91</v>
@@ -5378,17 +5378,17 @@
       <c r="A72" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" t="s">
         <v>18</v>
       </c>
       <c r="C72">
-        <v>65.349999999999994</v>
+        <v>65.55</v>
       </c>
       <c r="D72">
-        <v>70.95</v>
+        <v>71.150000000000006</v>
       </c>
       <c r="E72">
-        <v>77.05</v>
+        <v>77.25</v>
       </c>
       <c r="F72" s="3">
         <v>80</v>
@@ -5410,17 +5410,17 @@
       <c r="A73" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" t="s">
         <v>20</v>
       </c>
       <c r="C73">
-        <v>62.849999999999994</v>
+        <v>63.05</v>
       </c>
       <c r="D73">
-        <v>69.45</v>
+        <v>69.650000000000006</v>
       </c>
       <c r="E73">
-        <v>77.05</v>
+        <v>77.25</v>
       </c>
       <c r="F73" s="3">
         <v>72</v>
@@ -5442,17 +5442,17 @@
       <c r="A74" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" t="s">
         <v>11</v>
       </c>
       <c r="C74">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="D74">
-        <v>86.95</v>
+        <v>87.15</v>
       </c>
       <c r="E74">
-        <v>89.75</v>
+        <v>89.95</v>
       </c>
       <c r="F74" s="3">
         <v>97.2</v>
@@ -5474,17 +5474,17 @@
       <c r="A75" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" t="s">
         <v>13</v>
       </c>
       <c r="C75">
-        <v>81.75</v>
+        <v>81.95</v>
       </c>
       <c r="D75">
-        <v>84.95</v>
+        <v>85.15</v>
       </c>
       <c r="E75">
-        <v>88.15</v>
+        <v>88.350000000000009</v>
       </c>
       <c r="F75" s="3">
         <v>95.8</v>
@@ -5506,17 +5506,17 @@
       <c r="A76" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" t="s">
         <v>15</v>
       </c>
       <c r="C76">
-        <v>78.75</v>
+        <v>78.95</v>
       </c>
       <c r="D76">
-        <v>81.95</v>
+        <v>82.15</v>
       </c>
       <c r="E76">
-        <v>85.15</v>
+        <v>85.350000000000009</v>
       </c>
       <c r="F76" s="3">
         <v>92.8</v>
@@ -5538,17 +5538,17 @@
       <c r="A77" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" t="s">
         <v>16</v>
       </c>
       <c r="C77">
-        <v>69.349999999999994</v>
+        <v>69.55</v>
       </c>
       <c r="D77">
-        <v>74.95</v>
+        <v>75.150000000000006</v>
       </c>
       <c r="E77">
-        <v>81.05</v>
+        <v>81.25</v>
       </c>
       <c r="F77" s="3">
         <v>80</v>
@@ -5570,17 +5570,17 @@
       <c r="A78" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" t="s">
         <v>18</v>
       </c>
       <c r="C78">
-        <v>64.349999999999994</v>
+        <v>64.55</v>
       </c>
       <c r="D78">
-        <v>69.95</v>
+        <v>70.150000000000006</v>
       </c>
       <c r="E78">
-        <v>76.05</v>
+        <v>76.25</v>
       </c>
       <c r="F78" s="3">
         <v>70</v>
@@ -5602,17 +5602,17 @@
       <c r="A79" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" t="s">
         <v>20</v>
       </c>
       <c r="C79">
-        <v>61.849999999999994</v>
+        <v>62.05</v>
       </c>
       <c r="D79">
-        <v>68.45</v>
+        <v>68.650000000000006</v>
       </c>
       <c r="E79">
-        <v>76.05</v>
+        <v>76.25</v>
       </c>
       <c r="F79" s="3">
         <v>65</v>
@@ -5634,17 +5634,17 @@
       <c r="A80" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" t="s">
         <v>11</v>
       </c>
       <c r="C80">
-        <v>83.35</v>
+        <v>83.55</v>
       </c>
       <c r="D80">
-        <v>86.15</v>
+        <v>86.350000000000009</v>
       </c>
       <c r="E80">
-        <v>88.95</v>
+        <v>89.15</v>
       </c>
       <c r="F80" s="3">
         <v>96.8</v>
@@ -5666,17 +5666,17 @@
       <c r="A81" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" t="s">
         <v>13</v>
       </c>
       <c r="C81">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D81">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E81">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F81" s="3">
         <v>95</v>
@@ -5698,17 +5698,17 @@
       <c r="A82" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" t="s">
         <v>15</v>
       </c>
       <c r="C82">
-        <v>77.150000000000006</v>
+        <v>77.350000000000009</v>
       </c>
       <c r="D82">
-        <v>81.150000000000006</v>
+        <v>81.350000000000009</v>
       </c>
       <c r="E82">
-        <v>85.15</v>
+        <v>85.350000000000009</v>
       </c>
       <c r="F82" s="3">
         <v>91.5</v>
@@ -5730,17 +5730,17 @@
       <c r="A83" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" t="s">
         <v>16</v>
       </c>
       <c r="C83">
-        <v>68.55</v>
+        <v>68.75</v>
       </c>
       <c r="D83">
-        <v>74.150000000000006</v>
+        <v>74.350000000000009</v>
       </c>
       <c r="E83">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="F83" s="3">
         <v>79</v>
@@ -5762,17 +5762,17 @@
       <c r="A84" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" t="s">
         <v>18</v>
       </c>
       <c r="C84">
-        <v>62.55</v>
+        <v>62.75</v>
       </c>
       <c r="D84">
-        <v>69.150000000000006</v>
+        <v>69.350000000000009</v>
       </c>
       <c r="E84">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="F84" s="3">
         <v>68</v>
@@ -5794,17 +5794,17 @@
       <c r="A85" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" t="s">
         <v>20</v>
       </c>
       <c r="C85">
-        <v>61.05</v>
+        <v>61.25</v>
       </c>
       <c r="D85">
-        <v>67.650000000000006</v>
+        <v>67.850000000000009</v>
       </c>
       <c r="E85">
-        <v>75.25</v>
+        <v>75.45</v>
       </c>
       <c r="F85" s="3">
         <v>64</v>
@@ -5826,17 +5826,17 @@
       <c r="A86" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" t="s">
         <v>11</v>
       </c>
       <c r="C86">
-        <v>80.55</v>
+        <v>80.75</v>
       </c>
       <c r="D86">
-        <v>83.75</v>
+        <v>83.95</v>
       </c>
       <c r="E86">
-        <v>86.95</v>
+        <v>87.15</v>
       </c>
       <c r="F86" s="3">
         <v>95</v>
@@ -5858,17 +5858,17 @@
       <c r="A87" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" t="s">
         <v>13</v>
       </c>
       <c r="C87">
-        <v>80.55</v>
+        <v>80.75</v>
       </c>
       <c r="D87">
-        <v>83.75</v>
+        <v>83.95</v>
       </c>
       <c r="E87">
-        <v>86.95</v>
+        <v>87.15</v>
       </c>
       <c r="F87" s="3">
         <v>94</v>
@@ -5890,17 +5890,17 @@
       <c r="A88" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" t="s">
         <v>15</v>
       </c>
       <c r="C88">
-        <v>80.55</v>
+        <v>80.75</v>
       </c>
       <c r="D88">
-        <v>83.75</v>
+        <v>83.95</v>
       </c>
       <c r="E88">
-        <v>86.95</v>
+        <v>87.15</v>
       </c>
       <c r="F88" s="3">
         <v>94.5</v>
@@ -5922,17 +5922,17 @@
       <c r="A89" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" t="s">
         <v>16</v>
       </c>
       <c r="C89">
-        <v>66.150000000000006</v>
+        <v>66.350000000000009</v>
       </c>
       <c r="D89">
-        <v>71.75</v>
+        <v>71.95</v>
       </c>
       <c r="E89">
-        <v>77.849999999999994</v>
+        <v>78.05</v>
       </c>
       <c r="F89" s="3">
         <v>75</v>
@@ -5954,17 +5954,17 @@
       <c r="A90" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" t="s">
         <v>18</v>
       </c>
       <c r="C90">
-        <v>60.15</v>
+        <v>60.35</v>
       </c>
       <c r="D90">
-        <v>66.75</v>
+        <v>66.95</v>
       </c>
       <c r="E90">
-        <v>74.349999999999994</v>
+        <v>74.55</v>
       </c>
       <c r="F90" s="3">
         <v>65</v>
@@ -5986,17 +5986,17 @@
       <c r="A91" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="B91" t="s">
         <v>20</v>
       </c>
       <c r="C91">
-        <v>58.65</v>
+        <v>58.85</v>
       </c>
       <c r="D91">
-        <v>65.25</v>
+        <v>65.45</v>
       </c>
       <c r="E91">
-        <v>72.849999999999994</v>
+        <v>73.05</v>
       </c>
       <c r="F91" s="3">
         <v>60</v>
@@ -6018,17 +6018,17 @@
       <c r="A92" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="B92" t="s">
         <v>11</v>
       </c>
       <c r="C92">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D92">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E92">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F92" s="3">
         <v>94.5</v>
@@ -6050,17 +6050,17 @@
       <c r="A93" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B93" t="s">
         <v>13</v>
       </c>
       <c r="C93">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D93">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E93">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F93" s="3">
         <v>94.5</v>
@@ -6082,17 +6082,17 @@
       <c r="A94" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" t="s">
         <v>15</v>
       </c>
       <c r="C94">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D94">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E94">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F94" s="3">
         <v>94.5</v>
@@ -6114,17 +6114,17 @@
       <c r="A95" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B95" t="s">
         <v>16</v>
       </c>
       <c r="C95">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D95">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E95">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F95" s="3">
         <v>94.5</v>
@@ -6146,17 +6146,17 @@
       <c r="A96" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B96" t="s">
         <v>18</v>
       </c>
       <c r="C96">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D96">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E96">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F96" s="3">
         <v>94.5</v>
@@ -6178,17 +6178,17 @@
       <c r="A97" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B97" t="s">
         <v>20</v>
       </c>
       <c r="C97">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="D97">
-        <v>84.15</v>
+        <v>84.350000000000009</v>
       </c>
       <c r="E97">
-        <v>87.35</v>
+        <v>87.55</v>
       </c>
       <c r="F97" s="3">
         <v>94.5</v>
@@ -6210,17 +6210,17 @@
       <c r="A98" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" t="s">
         <v>11</v>
       </c>
       <c r="C98">
-        <v>80.349999999999994</v>
+        <v>80.55</v>
       </c>
       <c r="D98">
-        <v>83.55</v>
+        <v>83.75</v>
       </c>
       <c r="E98">
-        <v>86.75</v>
+        <v>86.95</v>
       </c>
       <c r="F98" s="3">
         <v>94.5</v>
@@ -6242,17 +6242,17 @@
       <c r="A99" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="B99" t="s">
         <v>13</v>
       </c>
       <c r="C99">
-        <v>77.55</v>
+        <v>77.75</v>
       </c>
       <c r="D99">
-        <v>81.55</v>
+        <v>81.75</v>
       </c>
       <c r="E99">
-        <v>85.55</v>
+        <v>85.75</v>
       </c>
       <c r="F99" s="3">
         <v>92</v>
@@ -6274,17 +6274,17 @@
       <c r="A100" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B100" s="2" t="s">
+      <c r="B100" t="s">
         <v>15</v>
       </c>
       <c r="C100">
-        <v>74.55</v>
+        <v>74.75</v>
       </c>
       <c r="D100">
-        <v>78.55</v>
+        <v>78.75</v>
       </c>
       <c r="E100">
-        <v>82.55</v>
+        <v>82.75</v>
       </c>
       <c r="F100" s="3">
         <v>86.5</v>
@@ -6306,17 +6306,17 @@
       <c r="A101" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B101" s="2" t="s">
+      <c r="B101" t="s">
         <v>16</v>
       </c>
       <c r="C101">
-        <v>65.95</v>
+        <v>66.150000000000006</v>
       </c>
       <c r="D101">
-        <v>71.55</v>
+        <v>71.75</v>
       </c>
       <c r="E101">
-        <v>77.650000000000006</v>
+        <v>77.850000000000009</v>
       </c>
       <c r="F101" s="3">
         <v>73</v>
@@ -6338,17 +6338,17 @@
       <c r="A102" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" t="s">
         <v>18</v>
       </c>
       <c r="C102">
-        <v>59.95</v>
+        <v>60.150000000000006</v>
       </c>
       <c r="D102">
-        <v>66.55</v>
+        <v>66.75</v>
       </c>
       <c r="E102">
-        <v>74.150000000000006</v>
+        <v>74.350000000000009</v>
       </c>
       <c r="F102" s="3">
         <v>62</v>
@@ -6370,17 +6370,17 @@
       <c r="A103" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="B103" t="s">
         <v>20</v>
       </c>
       <c r="C103">
-        <v>58.45</v>
+        <v>58.650000000000006</v>
       </c>
       <c r="D103">
-        <v>65.05</v>
+        <v>65.25</v>
       </c>
       <c r="E103">
-        <v>72.650000000000006</v>
+        <v>72.850000000000009</v>
       </c>
       <c r="F103" s="3">
         <v>58</v>
@@ -6402,17 +6402,17 @@
       <c r="A104" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B104" s="2" t="s">
+      <c r="B104" t="s">
         <v>11</v>
       </c>
       <c r="C104">
-        <v>80.05</v>
+        <v>80.25</v>
       </c>
       <c r="D104">
-        <v>83.25</v>
+        <v>83.45</v>
       </c>
       <c r="E104">
-        <v>86.45</v>
+        <v>86.65</v>
       </c>
       <c r="F104" s="3">
         <v>94</v>
@@ -6434,17 +6434,17 @@
       <c r="A105" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B105" s="2" t="s">
+      <c r="B105" t="s">
         <v>13</v>
       </c>
       <c r="C105">
-        <v>77.25</v>
+        <v>77.45</v>
       </c>
       <c r="D105">
-        <v>81.25</v>
+        <v>81.45</v>
       </c>
       <c r="E105">
-        <v>85.25</v>
+        <v>85.45</v>
       </c>
       <c r="F105" s="3">
         <v>91.5</v>
@@ -6466,17 +6466,17 @@
       <c r="A106" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="B106" t="s">
         <v>15</v>
       </c>
       <c r="C106">
-        <v>74.25</v>
+        <v>74.45</v>
       </c>
       <c r="D106">
-        <v>78.25</v>
+        <v>78.45</v>
       </c>
       <c r="E106">
-        <v>82.25</v>
+        <v>82.45</v>
       </c>
       <c r="F106" s="3">
         <v>85</v>
@@ -6498,17 +6498,17 @@
       <c r="A107" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B107" s="2" t="s">
+      <c r="B107" t="s">
         <v>16</v>
       </c>
       <c r="C107">
-        <v>65.650000000000006</v>
+        <v>65.850000000000009</v>
       </c>
       <c r="D107">
-        <v>71.25</v>
+        <v>71.45</v>
       </c>
       <c r="E107">
-        <v>77.349999999999994</v>
+        <v>77.55</v>
       </c>
       <c r="F107" s="3">
         <v>72</v>
@@ -6530,17 +6530,17 @@
       <c r="A108" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B108" s="2" t="s">
+      <c r="B108" t="s">
         <v>18</v>
       </c>
       <c r="C108">
-        <v>59.65</v>
+        <v>59.85</v>
       </c>
       <c r="D108">
-        <v>66.25</v>
+        <v>66.45</v>
       </c>
       <c r="E108">
-        <v>73.849999999999994</v>
+        <v>74.05</v>
       </c>
       <c r="F108" s="3">
         <v>60</v>
@@ -6562,17 +6562,17 @@
       <c r="A109" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="B109" t="s">
         <v>20</v>
       </c>
       <c r="C109">
-        <v>58.15</v>
+        <v>58.35</v>
       </c>
       <c r="D109">
-        <v>64.75</v>
+        <v>64.95</v>
       </c>
       <c r="E109">
-        <v>72.349999999999994</v>
+        <v>72.55</v>
       </c>
       <c r="F109" s="3">
         <v>56</v>
@@ -6594,17 +6594,17 @@
       <c r="A110" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="B110" t="s">
         <v>11</v>
       </c>
       <c r="C110">
-        <v>79.55</v>
+        <v>79.75</v>
       </c>
       <c r="D110">
-        <v>82.75</v>
+        <v>82.95</v>
       </c>
       <c r="E110">
-        <v>85.95</v>
+        <v>86.15</v>
       </c>
       <c r="F110" s="3">
         <v>94.2</v>
@@ -6626,17 +6626,17 @@
       <c r="A111" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="B111" t="s">
         <v>13</v>
       </c>
       <c r="C111">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D111">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E111">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F111" s="3">
         <v>92.5</v>
@@ -6658,17 +6658,17 @@
       <c r="A112" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B112" s="2" t="s">
+      <c r="B112" t="s">
         <v>15</v>
       </c>
       <c r="C112">
-        <v>73.75</v>
+        <v>73.95</v>
       </c>
       <c r="D112">
-        <v>77.75</v>
+        <v>77.95</v>
       </c>
       <c r="E112">
-        <v>81.75</v>
+        <v>81.95</v>
       </c>
       <c r="F112" s="3">
         <v>87</v>
@@ -6690,17 +6690,17 @@
       <c r="A113" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B113" s="2" t="s">
+      <c r="B113" t="s">
         <v>16</v>
       </c>
       <c r="C113">
-        <v>65.150000000000006</v>
+        <v>65.350000000000009</v>
       </c>
       <c r="D113">
-        <v>70.75</v>
+        <v>70.95</v>
       </c>
       <c r="E113">
-        <v>76.849999999999994</v>
+        <v>77.05</v>
       </c>
       <c r="F113" s="3">
         <v>75</v>
@@ -6722,17 +6722,17 @@
       <c r="A114" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B114" s="2" t="s">
+      <c r="B114" t="s">
         <v>18</v>
       </c>
       <c r="C114">
-        <v>59.15</v>
+        <v>59.35</v>
       </c>
       <c r="D114">
-        <v>65.75</v>
+        <v>65.95</v>
       </c>
       <c r="E114">
-        <v>73.349999999999994</v>
+        <v>73.55</v>
       </c>
       <c r="F114" s="3">
         <v>63</v>
@@ -6754,17 +6754,17 @@
       <c r="A115" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B115" s="2" t="s">
+      <c r="B115" t="s">
         <v>20</v>
       </c>
       <c r="C115">
-        <v>57.65</v>
+        <v>57.85</v>
       </c>
       <c r="D115">
-        <v>64.25</v>
+        <v>64.45</v>
       </c>
       <c r="E115">
-        <v>71.849999999999994</v>
+        <v>72.05</v>
       </c>
       <c r="F115" s="3">
         <v>60</v>
@@ -6786,17 +6786,17 @@
       <c r="A116" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B116" s="2" t="s">
+      <c r="B116" t="s">
         <v>11</v>
       </c>
       <c r="C116">
-        <v>76.95</v>
+        <v>77.150000000000006</v>
       </c>
       <c r="D116">
-        <v>80.95</v>
+        <v>81.150000000000006</v>
       </c>
       <c r="E116">
-        <v>84.95</v>
+        <v>85.15</v>
       </c>
       <c r="F116" s="3">
         <v>91.5</v>
@@ -6818,17 +6818,17 @@
       <c r="A117" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B117" s="2" t="s">
+      <c r="B117" t="s">
         <v>13</v>
       </c>
       <c r="C117">
-        <v>74.95</v>
+        <v>75.150000000000006</v>
       </c>
       <c r="D117">
-        <v>78.95</v>
+        <v>79.150000000000006</v>
       </c>
       <c r="E117">
-        <v>82.95</v>
+        <v>83.15</v>
       </c>
       <c r="F117" s="3">
         <v>88</v>
@@ -6850,17 +6850,17 @@
       <c r="A118" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B118" s="2" t="s">
+      <c r="B118" t="s">
         <v>15</v>
       </c>
       <c r="C118">
-        <v>71.95</v>
+        <v>72.150000000000006</v>
       </c>
       <c r="D118">
-        <v>75.95</v>
+        <v>76.150000000000006</v>
       </c>
       <c r="E118">
-        <v>79.95</v>
+        <v>80.150000000000006</v>
       </c>
       <c r="F118" s="3">
         <v>80</v>
@@ -6882,17 +6882,17 @@
       <c r="A119" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B119" s="2" t="s">
+      <c r="B119" t="s">
         <v>16</v>
       </c>
       <c r="C119">
-        <v>62.349999999999994</v>
+        <v>62.55</v>
       </c>
       <c r="D119">
-        <v>68.95</v>
+        <v>69.150000000000006</v>
       </c>
       <c r="E119">
-        <v>76.55</v>
+        <v>76.75</v>
       </c>
       <c r="F119" s="3">
         <v>66</v>
@@ -6914,17 +6914,17 @@
       <c r="A120" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B120" s="2" t="s">
+      <c r="B120" t="s">
         <v>18</v>
       </c>
       <c r="C120">
-        <v>57.35</v>
+        <v>57.550000000000004</v>
       </c>
       <c r="D120">
-        <v>63.95</v>
+        <v>64.150000000000006</v>
       </c>
       <c r="E120">
-        <v>71.55</v>
+        <v>71.75</v>
       </c>
       <c r="F120" s="3">
         <v>55</v>
@@ -6946,17 +6946,17 @@
       <c r="A121" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="B121" t="s">
         <v>20</v>
       </c>
       <c r="C121">
-        <v>55.85</v>
+        <v>56.050000000000004</v>
       </c>
       <c r="D121">
-        <v>62.45</v>
+        <v>62.650000000000006</v>
       </c>
       <c r="E121">
-        <v>70.05</v>
+        <v>70.25</v>
       </c>
       <c r="F121" s="3">
         <v>52</v>
@@ -6978,17 +6978,17 @@
       <c r="A122" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B122" t="s">
         <v>11</v>
       </c>
       <c r="C122">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D122">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E122">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F122" s="3">
         <v>89</v>
@@ -7010,17 +7010,17 @@
       <c r="A123" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B123" s="2" t="s">
+      <c r="B123" t="s">
         <v>13</v>
       </c>
       <c r="C123">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D123">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E123">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F123" s="3">
         <v>89</v>
@@ -7042,17 +7042,17 @@
       <c r="A124" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B124" s="2" t="s">
+      <c r="B124" t="s">
         <v>15</v>
       </c>
       <c r="C124">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D124">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E124">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F124" s="3">
         <v>89</v>
@@ -7074,17 +7074,17 @@
       <c r="A125" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B125" s="2" t="s">
+      <c r="B125" t="s">
         <v>16</v>
       </c>
       <c r="C125">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D125">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E125">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F125" s="3">
         <v>89</v>
@@ -7106,17 +7106,17 @@
       <c r="A126" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B126" s="2" t="s">
+      <c r="B126" t="s">
         <v>18</v>
       </c>
       <c r="C126">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D126">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E126">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F126" s="3">
         <v>89</v>
@@ -7138,17 +7138,17 @@
       <c r="A127" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B127" s="2" t="s">
+      <c r="B127" t="s">
         <v>20</v>
       </c>
       <c r="C127">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="D127">
-        <v>80.75</v>
+        <v>80.95</v>
       </c>
       <c r="E127">
-        <v>84.75</v>
+        <v>84.95</v>
       </c>
       <c r="F127" s="3">
         <v>89</v>
@@ -7170,17 +7170,17 @@
       <c r="A128" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B128" s="2" t="s">
+      <c r="B128" t="s">
         <v>11</v>
       </c>
       <c r="C128">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D128">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E128">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F128" s="3">
         <v>90</v>
@@ -7202,17 +7202,17 @@
       <c r="A129" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B129" s="2" t="s">
+      <c r="B129" t="s">
         <v>13</v>
       </c>
       <c r="C129">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D129">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E129">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F129" s="3">
         <v>88</v>
@@ -7234,17 +7234,17 @@
       <c r="A130" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" t="s">
         <v>15</v>
       </c>
       <c r="C130">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D130">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E130">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F130" s="3">
         <v>85</v>
@@ -7266,17 +7266,17 @@
       <c r="A131" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B131" s="2" t="s">
+      <c r="B131" t="s">
         <v>16</v>
       </c>
       <c r="C131">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D131">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E131">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F131" s="3">
         <v>72</v>
@@ -7298,17 +7298,17 @@
       <c r="A132" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B132" t="s">
         <v>18</v>
       </c>
       <c r="C132">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D132">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E132">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F132" s="3">
         <v>60</v>
@@ -7330,17 +7330,17 @@
       <c r="A133" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B133" s="2" t="s">
+      <c r="B133" t="s">
         <v>20</v>
       </c>
       <c r="C133">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="D133">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="E133">
-        <v>84.25</v>
+        <v>84.45</v>
       </c>
       <c r="F133" s="3">
         <v>58</v>
@@ -7362,17 +7362,17 @@
       <c r="A134" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B134" t="s">
         <v>11</v>
       </c>
       <c r="C134">
-        <v>72.25</v>
+        <v>72.45</v>
       </c>
       <c r="D134">
-        <v>76.25</v>
+        <v>76.45</v>
       </c>
       <c r="E134">
-        <v>80.25</v>
+        <v>80.45</v>
       </c>
       <c r="F134" s="3">
         <v>82</v>
@@ -7394,17 +7394,17 @@
       <c r="A135" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B135" s="2" t="s">
+      <c r="B135" t="s">
         <v>13</v>
       </c>
       <c r="C135">
-        <v>69.25</v>
+        <v>69.45</v>
       </c>
       <c r="D135">
-        <v>74.25</v>
+        <v>74.45</v>
       </c>
       <c r="E135">
-        <v>79.75</v>
+        <v>79.95</v>
       </c>
       <c r="F135" s="3">
         <v>78</v>
@@ -7426,17 +7426,17 @@
       <c r="A136" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B136" s="2" t="s">
+      <c r="B136" t="s">
         <v>15</v>
       </c>
       <c r="C136">
-        <v>66.25</v>
+        <v>66.45</v>
       </c>
       <c r="D136">
-        <v>71.25</v>
+        <v>71.45</v>
       </c>
       <c r="E136">
-        <v>76.75</v>
+        <v>76.95</v>
       </c>
       <c r="F136" s="3">
         <v>72</v>
@@ -7458,17 +7458,17 @@
       <c r="A137" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B137" s="2" t="s">
+      <c r="B137" t="s">
         <v>16</v>
       </c>
       <c r="C137">
-        <v>57.65</v>
+        <v>57.85</v>
       </c>
       <c r="D137">
-        <v>64.25</v>
+        <v>64.45</v>
       </c>
       <c r="E137">
-        <v>71.849999999999994</v>
+        <v>72.05</v>
       </c>
       <c r="F137" s="3">
         <v>60</v>
@@ -7490,17 +7490,17 @@
       <c r="A138" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B138" t="s">
         <v>18</v>
       </c>
       <c r="C138">
-        <v>52.65</v>
+        <v>52.85</v>
       </c>
       <c r="D138">
-        <v>59.25</v>
+        <v>59.45</v>
       </c>
       <c r="E138">
-        <v>66.849999999999994</v>
+        <v>67.05</v>
       </c>
       <c r="F138" s="3">
         <v>50</v>
@@ -7522,17 +7522,17 @@
       <c r="A139" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B139" s="2" t="s">
+      <c r="B139" t="s">
         <v>20</v>
       </c>
       <c r="C139">
-        <v>51.15</v>
+        <v>51.35</v>
       </c>
       <c r="D139">
-        <v>57.75</v>
+        <v>57.95</v>
       </c>
       <c r="E139">
-        <v>65.349999999999994</v>
+        <v>65.55</v>
       </c>
       <c r="F139" s="3">
         <v>48</v>
@@ -7554,17 +7554,17 @@
       <c r="A140" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B140" s="2" t="s">
+      <c r="B140" t="s">
         <v>11</v>
       </c>
       <c r="C140">
-        <v>64.75</v>
+        <v>64.95</v>
       </c>
       <c r="D140">
-        <v>69.75</v>
+        <v>69.95</v>
       </c>
       <c r="E140">
-        <v>75.25</v>
+        <v>75.45</v>
       </c>
       <c r="F140" s="3">
         <v>70</v>
@@ -7586,17 +7586,17 @@
       <c r="A141" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="B141" t="s">
         <v>13</v>
       </c>
       <c r="C141">
-        <v>61.75</v>
+        <v>61.95</v>
       </c>
       <c r="D141">
-        <v>67.75</v>
+        <v>67.95</v>
       </c>
       <c r="E141">
-        <v>74.75</v>
+        <v>74.95</v>
       </c>
       <c r="F141" s="3">
         <v>66</v>
@@ -7618,17 +7618,17 @@
       <c r="A142" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B142" t="s">
         <v>15</v>
       </c>
       <c r="C142">
-        <v>58.75</v>
+        <v>58.95</v>
       </c>
       <c r="D142">
-        <v>64.75</v>
+        <v>64.95</v>
       </c>
       <c r="E142">
-        <v>71.75</v>
+        <v>71.95</v>
       </c>
       <c r="F142" s="3">
         <v>60</v>
@@ -7650,17 +7650,17 @@
       <c r="A143" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B143" s="2" t="s">
+      <c r="B143" t="s">
         <v>16</v>
       </c>
       <c r="C143">
-        <v>51.15</v>
+        <v>51.35</v>
       </c>
       <c r="D143">
-        <v>57.75</v>
+        <v>57.95</v>
       </c>
       <c r="E143">
-        <v>65.349999999999994</v>
+        <v>65.55</v>
       </c>
       <c r="F143" s="3">
         <v>48</v>
@@ -7682,17 +7682,17 @@
       <c r="A144" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="B144" t="s">
         <v>18</v>
       </c>
       <c r="C144">
-        <v>46.15</v>
+        <v>46.35</v>
       </c>
       <c r="D144">
-        <v>52.75</v>
+        <v>52.95</v>
       </c>
       <c r="E144">
-        <v>60.35</v>
+        <v>60.550000000000004</v>
       </c>
       <c r="F144" s="3">
         <v>40</v>
@@ -7714,17 +7714,17 @@
       <c r="A145" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B145" t="s">
         <v>20</v>
       </c>
       <c r="C145">
-        <v>44.65</v>
+        <v>44.85</v>
       </c>
       <c r="D145">
-        <v>51.25</v>
+        <v>51.45</v>
       </c>
       <c r="E145">
-        <v>58.85</v>
+        <v>59.050000000000004</v>
       </c>
       <c r="F145" s="3">
         <v>40</v>

</xml_diff>